<commit_message>
Update the data sheet
</commit_message>
<xml_diff>
--- a/data/Hindcon_specility_TDS_MSDS.xlsx
+++ b/data/Hindcon_specility_TDS_MSDS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="69">
   <si>
     <t>ALPHA SET PRO tds-speciality NEW</t>
   </si>
@@ -210,13 +210,34 @@
   </si>
   <si>
     <t>HC019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALPHA SET </t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLD BOX </t>
+  </si>
+  <si>
+    <t>SHELL RESIN</t>
+  </si>
+  <si>
+    <t>FURAN RESIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOLID PF RESIN </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACID CURE </t>
+  </si>
+  <si>
+    <t>HC020</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -232,14 +253,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -249,7 +262,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -257,23 +270,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -552,30 +576,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="3"/>
-    <col min="2" max="2" width="18.5703125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="18.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="49.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="90" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="107.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -583,6 +607,9 @@
       <c r="A2" s="3" t="s">
         <v>43</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>62</v>
+      </c>
       <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
@@ -594,6 +621,9 @@
       <c r="A3" s="3" t="s">
         <v>44</v>
       </c>
+      <c r="B3" s="1" t="s">
+        <v>63</v>
+      </c>
       <c r="C3" s="1" t="s">
         <v>2</v>
       </c>
@@ -605,6 +635,9 @@
       <c r="A4" s="3" t="s">
         <v>45</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
@@ -616,6 +649,9 @@
       <c r="A5" s="3" t="s">
         <v>46</v>
       </c>
+      <c r="B5" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="C5" s="1" t="s">
         <v>6</v>
       </c>
@@ -627,6 +663,9 @@
       <c r="A6" s="3" t="s">
         <v>47</v>
       </c>
+      <c r="B6" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
@@ -638,6 +677,9 @@
       <c r="A7" s="3" t="s">
         <v>48</v>
       </c>
+      <c r="B7" s="1" t="s">
+        <v>67</v>
+      </c>
       <c r="C7" s="1" t="s">
         <v>10</v>
       </c>
@@ -649,150 +691,191 @@
       <c r="A8" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>26</v>
+      <c r="B9" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>27</v>
+      <c r="B10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
+      <c r="B11" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>29</v>
+      <c r="B12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>30</v>
+      <c r="B13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>31</v>
+      <c r="B14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>32</v>
+      <c r="B15" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>33</v>
+      <c r="B16" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>34</v>
+      <c r="B17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>35</v>
+      <c r="B18" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>36</v>
+      <c r="B19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="B20" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="E21" s="1" t="s">
         <v>37</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E13" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>